<commit_message>
scan: seg6 2026-10-09 00:27 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq7_2026-10-08.xlsx
+++ b/output/full_scan/batch_seq7_2026-10-08.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>77.98117719073518</v>
+        <v>77.98117717601194</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>32.15654620909395</v>
+        <v>32.15654623362533</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>4.677801058886754</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>3.628760469657844</v>
+        <v>3.628760469858125</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>74.83919999967526</v>
+        <v>74.83919994575774</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>31.18927916537371</v>
+        <v>31.18927914586173</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>8.986045869853438</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>0.3697256364365203</v>
+        <v>0.369725636302992</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>72.28893207205387</v>
+        <v>72.28893200630961</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>34.97202336126707</v>
+        <v>34.97202339169168</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>3.600972489894296</v>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>72.69184579894349</v>
+        <v>72.69184569411291</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>45.21680537757569</v>
+        <v>45.21680541636936</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>1.588509040452033</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>1.844335490855054</v>
+        <v>1.844335491300137</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>61.29899891042768</v>
+        <v>61.29899892586664</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>19.84932216453936</v>
+        <v>19.84932217075763</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>1.958211046203465</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.1140782877735906</v>
+        <v>0.1140782857706945</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>67.31496915551332</v>
+        <v>67.31496915714027</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>43.77619171200405</v>
+        <v>43.7761917226742</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>2.234766192675654</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>1.698063411885382</v>
+        <v>1.698063411896504</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>956.6378137424812</v>
+        <v>956.637813742482</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>61.3</v>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>62.92622618335086</v>
+        <v>62.92622639186504</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>31.60847789408559</v>
+        <v>31.60847791229341</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>5.004460398320227</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.1403973477637987</v>
+        <v>0.1403973477860597</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>78.2648912943897</v>
+        <v>78.26489127375122</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>58.86761665530558</v>
+        <v>58.86761669835523</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>1.407805070964943</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>1.694036728375709</v>
+        <v>1.694036728498101</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>62.05634853406622</v>
+        <v>62.05634877219592</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>23.72131104997342</v>
+        <v>23.7213110707453</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>4.925135988513275</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.0804040785561031</v>
+        <v>0.0804040784448317</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>72.16885567686451</v>
+        <v>72.16885568885512</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>34.46886449653184</v>
+        <v>34.46886449653183</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>0.9899212603935608</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>17.23845899032295</v>
+        <v>17.23845899121328</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>67.04068619922376</v>
+        <v>67.04068626206461</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>49.95145011754379</v>
+        <v>49.95145008508936</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>0.9765676066623864</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>0.1804956501168209</v>
+        <v>0.1804956500723107</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1121,7 +1121,7 @@
         <v/>
       </c>
       <c r="D13" s="2" t="n">
-        <v>839.1880866732728</v>
+        <v>839.1880866732723</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>1130</v>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>60.07551026753651</v>
+        <v>60.07551026141745</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>21.40133738518623</v>
+        <v>21.40133734888824</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>1.558748156782288</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>25.88294477089338</v>
+        <v>25.88294477167234</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>60.98143055668546</v>
+        <v>60.98143054996154</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>34.82024462389591</v>
+        <v>34.82024472648525</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>0.4722500484871325</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>2.933073678173151</v>
+        <v>2.933073678262178</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>59.93141592618346</v>
+        <v>59.93141592953386</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>29.97730853597498</v>
+        <v>29.97730848545966</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>0.4599786403510817</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0.7378369567426972</v>
+        <v>0.7378369566981888</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1280,7 +1280,7 @@
         <v/>
       </c>
       <c r="D16" s="2" t="n">
-        <v>812.0413633490103</v>
+        <v>812.0413633490097</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>57.9</v>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>63.85340559431072</v>
+        <v>63.85340557227724</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>52.76980735254075</v>
+        <v>52.76980748079333</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>0.7579383884849463</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.5398678628627822</v>
+        <v>0.5398678632856089</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>62.45087865278765</v>
+        <v>62.45087865496363</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>37.42512655896412</v>
+        <v>37.4251265617586</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.6671479768843608</v>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>53.74423830941075</v>
+        <v>53.74423820228884</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>16.77141116494179</v>
+        <v>16.77141114280965</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>3.369596032338268</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>1.821047945797788</v>
+        <v>1.821047945352711</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1439,7 +1439,7 @@
         <v/>
       </c>
       <c r="D19" s="2" t="n">
-        <v>784.4836227024334</v>
+        <v>784.4836227024335</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>94.5</v>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>64.7112899571481</v>
+        <v>64.71129052355218</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>21.70001782748222</v>
+        <v>21.7000178768023</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>3.412775877263639</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>0.55956369351113</v>
+        <v>0.5595636934888701</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>59.92352121011447</v>
+        <v>59.92352121230864</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>28.10003333987877</v>
+        <v>28.10003335483679</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>0.5938275576627133</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>4.510599067805451</v>
+        <v>4.510599067694205</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1562,7 +1562,7 @@
         <v>58.98838755467104</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>19.98650735814681</v>
+        <v>19.98650739552722</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>0.9086385847321282</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>0.6291563055549811</v>
+        <v>0.6291563055438465</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>60.35221765198232</v>
+        <v>60.35221769892848</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>22.91547818199159</v>
+        <v>22.91547816282246</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>0.7168845755629784</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0.0546352422759546</v>
+        <v>0.054635242231444</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>84.81904247773085</v>
+        <v>84.81904218199512</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>39.87560954545664</v>
+        <v>39.8756095946842</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>1.427086274795852</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0.5232259807619064</v>
+        <v>0.5232259810734681</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>57.21265621380266</v>
+        <v>57.21265625371881</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>22.19883912550189</v>
+        <v>22.198839170357</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>1.263692939504653</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.5573243875192722</v>
+        <v>0.5573243875637813</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1757,7 +1757,7 @@
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>695.1341194009377</v>
+        <v>695.1341194009391</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>373.5</v>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>57.69248778392433</v>
+        <v>57.69248789179114</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>19.90899441022736</v>
+        <v>19.90899441238585</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0.6487988894853873</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>3.143409793946931</v>
+        <v>3.143409793613073</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>55.8933995293924</v>
+        <v>55.89339953111688</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>45.23997928310471</v>
+        <v>45.23997928287091</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>1.273289781574087</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.3979803102985997</v>
+        <v>0.3979803101205723</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>50.80152832061761</v>
+        <v>50.80152832275295</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>42.73984061694701</v>
+        <v>42.73984061532882</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>2.70371125986594</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>-14.59945755964882</v>
+        <v>-14.5994575598046</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>62.91383970602699</v>
+        <v>62.91383970364562</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>37.93571632168664</v>
+        <v>37.93571629859821</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>1.81992411117357</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>1.511951910761302</v>
+        <v>1.511951910716803</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>57.31869471152243</v>
+        <v>57.31869469677081</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>51.64979245952407</v>
+        <v>51.64979246264099</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>0.2074449238610302</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>-0.4748035917449682</v>
+        <v>-0.474803591611451</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2022,7 +2022,7 @@
         <v/>
       </c>
       <c r="D30" s="2" t="n">
-        <v>643.286952833548</v>
+        <v>643.2869528335478</v>
       </c>
       <c r="E30" s="2" t="n">
         <v>375.5</v>
@@ -2039,7 +2039,7 @@
         <v>63.00320033927046</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>20.37663348660539</v>
+        <v>20.37663348387723</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>3.292200462809101</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>5.279758642790048</v>
+        <v>5.279758642122435</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>56.78172333427752</v>
+        <v>56.78172321453793</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>24.24039645038262</v>
+        <v>24.24039646995633</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>1.222391606073116</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.0949734364634701</v>
+        <v>0.0949734366415035</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>53.51323026522572</v>
+        <v>53.51323021848238</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>29.13121616453397</v>
+        <v>29.13121614428152</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>1.035954040179551</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-1.002055784747014</v>
+        <v>-1.002055784524414</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>52.31230420162523</v>
+        <v>52.31230419904265</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>15.24503772292839</v>
+        <v>15.24503784538327</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.9618356769682858</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>2.330839335517688</v>
+        <v>2.330839334404953</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2234,7 +2234,7 @@
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>613.0533900657981</v>
+        <v>613.053390065798</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>481</v>
@@ -2248,7 +2248,7 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>55.80179142974355</v>
+        <v>55.80179150525545</v>
       </c>
       <c r="I34" s="2" t="n">
         <v>18.26107891569308</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>1.87820560922014</v>
+        <v>1.878205608663809</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>611.5031678694775</v>
+        <v>611.5031678694868</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>25.1</v>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>52.93022549832351</v>
+        <v>52.93022559344925</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>25.70036322992832</v>
+        <v>25.70036353326663</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.6387597636512786</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.145381293541036</v>
+        <v>0.1453812940973958</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>50.31989706546384</v>
+        <v>50.31989693771708</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>31.21094354017633</v>
+        <v>31.21094350049081</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.4090974794755025</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-0.9230504694801738</v>
+        <v>-0.923050468100402</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2393,7 +2393,7 @@
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>598.4885307453976</v>
+        <v>598.4885307453978</v>
       </c>
       <c r="E37" s="2" t="n">
         <v>3320</v>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>54.38830474558928</v>
+        <v>54.38830474779282</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>20.54630198732726</v>
+        <v>20.54630192904309</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>1.474164731532992</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>-38.65873844289933</v>
+        <v>-38.65873843399758</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>55.74044005177391</v>
+        <v>55.74044001556322</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>22.01416928547598</v>
+        <v>22.01416930767322</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.2994834962647691</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>0.8141755918967528</v>
+        <v>0.8141755920302727</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>70.10524082817399</v>
+        <v>70.10524096242435</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>39.87952338650506</v>
+        <v>39.87952354928882</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.2721303613979708</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>0.0660485991336099</v>
+        <v>0.0660485988888147</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>54.44282150031537</v>
+        <v>54.44282154055057</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>35.68922854955495</v>
+        <v>35.68922857887784</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>1.034954254007886</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>-17.7772750274648</v>
+        <v>-17.77727502969026</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>66.94144635673362</v>
+        <v>66.94144622262783</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>33.9762935339493</v>
+        <v>33.976293537517</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.9702302192733628</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0.7057447906471799</v>
+        <v>0.70574479069169</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>49.69337062924125</v>
+        <v>49.69337066999818</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>23.60458250174502</v>
+        <v>23.60458249324902</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.4012323580511459</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-5.50905429970808</v>
+        <v>-5.509054300153176</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>54.23871075365391</v>
+        <v>54.23871078293885</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>34.77611100972021</v>
+        <v>34.7761110393562</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.4059126960222002</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>0.4189830323653893</v>
+        <v>0.4189830296948678</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2764,7 +2764,7 @@
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>546.2834860411059</v>
+        <v>546.2834860411032</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>32.05</v>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>60.39992763303238</v>
+        <v>60.39992765887241</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>20.71831703474518</v>
+        <v>20.71831704960949</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.76842308365379</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.1499796471691652</v>
+        <v>0.1499796471914191</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>53.33818506968817</v>
+        <v>53.33818508233588</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>21.31535232268809</v>
+        <v>21.3153523464286</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.5655523515812341</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-0.1159263829590788</v>
+        <v>-0.1159263832261293</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>52.02230678942315</v>
+        <v>52.02230678844378</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>11.11308168167067</v>
+        <v>11.1130816851763</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>2.418127818287665</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>3.409480480128253</v>
+        <v>3.409480480239531</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>51.56681847522092</v>
+        <v>51.56681841409393</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>17.15662838813007</v>
+        <v>17.15662840939718</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>2.372104056297936</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.0356306632060784</v>
+        <v>0.0356306631393133</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2993,7 +2993,7 @@
         <v>50.90533411562049</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>11.92475895729071</v>
+        <v>11.92475909126024</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>2.690725197121355</v>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>31.69493958808852</v>
+        <v>31.69496352542404</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>32.59385518904277</v>
+        <v>32.59382456590205</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>2.013053626871306</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.411281829574265</v>
+        <v>0.4112815436474344</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>51.97356044181092</v>
+        <v>51.97356043739259</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>25.38572039941569</v>
+        <v>25.3857206679741</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.3049131851882646</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>0.0996167199309265</v>
+        <v>0.0996167198419399</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>59.58064841344882</v>
+        <v>59.58064851185962</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>19.58274032691225</v>
+        <v>19.58274036768908</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>1.384728293230064</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-0.0258894578160754</v>
+        <v>-0.0258894578383286</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>48.30777086673174</v>
+        <v>48.30777085804998</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>20.42390698323611</v>
+        <v>20.42390699357122</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.3048159697488382</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-0.9461648875705762</v>
+        <v>-0.9461648875038152</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>44.60397902113559</v>
+        <v>44.60397899676303</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>20.06361047896212</v>
+        <v>20.06361044251097</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>1.657099006575845</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-0.018381586220308</v>
+        <v>-0.0183815861758046</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3294,7 +3294,7 @@
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>516.5411916125166</v>
+        <v>516.541191612517</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>34</v>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>52.12373603434921</v>
+        <v>52.12373603468044</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>12.51999808499355</v>
+        <v>12.51999809700345</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>4.697438928066099</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-0.388562942987031</v>
+        <v>-0.3885629429981603</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3347,7 +3347,7 @@
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>499.8940287804555</v>
+        <v>499.8940287804564</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>31.8</v>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>55.58318130453939</v>
+        <v>55.58318128188915</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>13.61404875029658</v>
+        <v>13.61404865239989</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>2.522669972002799</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.0809028409738967</v>
+        <v>0.0809028410406602</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>52.08940428419049</v>
+        <v>52.08940430090089</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>8.136581864613728</v>
+        <v>8.136581882106729</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.6762794966548318</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.1599916667316492</v>
+        <v>0.1599916666871392</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3453,7 +3453,7 @@
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>497.7344371837372</v>
+        <v>497.7344371837373</v>
       </c>
       <c r="E57" s="2" t="n">
         <v>308.5</v>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>39.43794983377514</v>
+        <v>39.43794979259269</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>20.72798230115453</v>
+        <v>20.72798244324854</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>1.787865829468616</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.3012250303597303</v>
+        <v>0.3012250305823132</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>51.5001806545109</v>
+        <v>51.50018067503167</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>14.47981325637352</v>
+        <v>14.47981322996224</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>1.258746950402002</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.4586355739613266</v>
+        <v>0.4586355738945528</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>56.76519324867839</v>
+        <v>56.76519303941593</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>35.5907117403283</v>
+        <v>35.59071161988214</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>0.3036177039866246</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.5808116665808498</v>
+        <v>-0.5808116651343025</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>46.44390457755065</v>
+        <v>46.44390463852518</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>10.22681461972178</v>
+        <v>10.22681481625967</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.4974877860698913</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.4033154440088333</v>
+        <v>-0.4033154453440959</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3665,7 +3665,7 @@
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>445.2297543505235</v>
+        <v>445.2297543505237</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>53</v>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>54.9499842260415</v>
+        <v>54.94998433308984</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>12.37374615186898</v>
+        <v>12.37374604800107</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.7058512164653069</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.1118318262250934</v>
+        <v>0.1118318260248105</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>42.65358382213411</v>
+        <v>42.65358391383797</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>16.43027827107189</v>
+        <v>16.43027833260744</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.4514499282606705</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.0176192468611204</v>
+        <v>0.017619246838868</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3771,7 +3771,7 @@
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>444.0379372480065</v>
+        <v>444.0379372480064</v>
       </c>
       <c r="E63" s="2" t="n">
         <v>138</v>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>52.46872792007832</v>
+        <v>52.46872791315004</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>14.33720509509919</v>
+        <v>14.33720508707962</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.9173885250808316</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>1.306738551555575</v>
+        <v>1.306738551711339</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>71.45298382247145</v>
+        <v>71.4529838752851</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>33.66978101331799</v>
+        <v>33.66978099130186</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.6454769209701262</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.4994493593467561</v>
+        <v>0.4994493591701809</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>49.87765929698684</v>
+        <v>49.87765930767628</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>13.34529037380726</v>
+        <v>13.34529036475397</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.9913914097643453</v>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>48.63256509577737</v>
+        <v>48.63256502103121</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>16.96765015565864</v>
+        <v>16.96765016338534</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.4202645054255581</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-1.896940140077733</v>
+        <v>-1.896940139632627</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3983,7 +3983,7 @@
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>427.7459199084133</v>
+        <v>427.7459199084135</v>
       </c>
       <c r="E67" s="2" t="n">
         <v>1050</v>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>45.53960809113265</v>
+        <v>45.53960811224642</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>19.34935631695816</v>
+        <v>19.3493563504213</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.4803562824736629</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-5.711683038962994</v>
+        <v>-5.711683043636535</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>32.04679702300979</v>
+        <v>32.04679708368592</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>44.11891516341322</v>
+        <v>44.11891517530357</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.6863659101217567</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>148.6955938269323</v>
+        <v>148.6955938158051</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4089,7 +4089,7 @@
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>422.9168282810194</v>
+        <v>422.9168282810193</v>
       </c>
       <c r="E69" s="2" t="n">
         <v>99.2</v>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>32.77380213114456</v>
+        <v>32.77380206114455</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>32.08668485378289</v>
+        <v>32.08668489455518</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>4.026592479560937</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.1379847759255845</v>
+        <v>0.1379847763039099</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>31.79771761897067</v>
+        <v>31.7977173726148</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>29.1483098406514</v>
+        <v>29.14830981818112</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>1.73602479466562</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.345219976349151</v>
+        <v>-0.3452199761043486</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4195,7 +4195,7 @@
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>399.6809458718941</v>
+        <v>399.6809458718973</v>
       </c>
       <c r="E71" s="2" t="n">
         <v>44.9</v>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>59.30997280335322</v>
+        <v>59.3099726755714</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>27.58468479194518</v>
+        <v>27.58468502559269</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.4062291653049218</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.5978495107879856</v>
+        <v>0.5978495108324979</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4248,7 +4248,7 @@
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>398.8761491707785</v>
+        <v>398.8761491707783</v>
       </c>
       <c r="E72" s="2" t="n">
         <v>48.05</v>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>48.7185650015343</v>
+        <v>48.7185649513577</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>26.7220687539976</v>
+        <v>26.72206878919548</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.321676861844581</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.027659345543632</v>
+        <v>-0.0276593456994057</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>56.7869893579715</v>
+        <v>56.7869892741137</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>18.62629735919673</v>
+        <v>18.62629727608011</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.9010651670525968</v>
@@ -4354,7 +4354,7 @@
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>372.3149657976856</v>
+        <v>372.3149657976858</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>63.8</v>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>50.23996945873404</v>
+        <v>50.2399688689736</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>21.76144600847763</v>
+        <v>21.76144599795549</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.6924347398800291</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.3768378598142667</v>
+        <v>0.3768378602593487</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4407,7 +4407,7 @@
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>371.8250068266359</v>
+        <v>371.8250068266358</v>
       </c>
       <c r="E75" s="2" t="n">
         <v>1020</v>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>46.43350837535134</v>
+        <v>46.43350865589453</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>9.953467438189769</v>
+        <v>9.95346746950699</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>1.114669928673481</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>3.399155881748182</v>
+        <v>3.399155882860882</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>43.93109222988586</v>
+        <v>43.93109224022478</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>17.17684108014084</v>
+        <v>17.17684093117329</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.5066068051551553</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>0.0347559544363359</v>
+        <v>0.0347559546232736</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>49.14628568085883</v>
+        <v>49.146285629745</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>14.23185935039161</v>
+        <v>14.23185934882007</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>1.082389298403912</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.0431989902253679</v>
+        <v>0.0431989906704554</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4566,7 +4566,7 @@
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>369.483523386737</v>
+        <v>369.4835233867393</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>476</v>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>35.74053649779979</v>
+        <v>35.74053652099506</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>24.98249141930964</v>
+        <v>24.98249145296979</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>2.2835170369843</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.9431394308956484</v>
+        <v>0.943139429560386</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>45.72344529133213</v>
+        <v>45.72344533501381</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>22.91381087600315</v>
+        <v>22.91381087841981</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.112792326522207</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.3960621067801096</v>
+        <v>-0.3960621071361779</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4672,7 +4672,7 @@
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>356.1528024815279</v>
+        <v>356.1528024815327</v>
       </c>
       <c r="E80" s="2" t="n">
         <v>41.8</v>
@@ -4686,7 +4686,7 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>40.42784767701897</v>
+        <v>40.42784782528297</v>
       </c>
       <c r="I80" s="2" t="n">
         <v>28.2648153374927</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-0.112371955306505</v>
+        <v>-0.1123719555735493</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4725,7 +4725,7 @@
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>354.412218611817</v>
+        <v>354.4122186118169</v>
       </c>
       <c r="E81" s="2" t="n">
         <v>1080</v>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>47.17907478357301</v>
+        <v>47.17907481520366</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>10.44503000443969</v>
+        <v>10.4450300044397</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.4386535314835921</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-5.777790600725043</v>
+        <v>-5.777790601948931</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>49.97945207804331</v>
+        <v>49.97945205825455</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>11.84312292544474</v>
+        <v>11.84312293151415</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>0.4282696609609741</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.1079734458387487</v>
+        <v>0.1079734457719877</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>48.93378327963145</v>
+        <v>48.93378349139741</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>17.03167714343159</v>
+        <v>17.03167715970389</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.5063964740271319</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.0718074553347255</v>
+        <v>0.0718074553792336</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4901,7 +4901,7 @@
         <v>50.36687054060497</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>6.867971321887838</v>
+        <v>6.867971449404723</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>1.23093580121998</v>
@@ -4937,7 +4937,7 @@
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>337.5790327226554</v>
+        <v>337.5790327226318</v>
       </c>
       <c r="E85" s="2" t="n">
         <v>41.55</v>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>52.02671478080331</v>
+        <v>52.02671497220875</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>17.52343363554183</v>
+        <v>17.52343362253448</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>0.7005465057417336</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>0.0694930731810133</v>
+        <v>0.0694930730474904</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -4990,7 +4990,7 @@
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>336.2429150946989</v>
+        <v>336.2429150946988</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>1415</v>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>47.65097967232668</v>
+        <v>47.65097970079854</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>16.83326265983093</v>
+        <v>16.8332625949138</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.4293236982277061</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-22.49594668519212</v>
+        <v>-22.49594668619365</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>46.65280280926062</v>
+        <v>46.65280283291249</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>13.43740418511641</v>
+        <v>13.43740418864064</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.6148936400018552</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.5909126819564725</v>
+        <v>0.5909126842931918</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>50.18046390548595</v>
+        <v>50.18046394032337</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>23.36733373073475</v>
+        <v>23.36733376986713</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>1.057565219358469</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.0697857836479558</v>
+        <v>0.06978578344767331</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5166,7 +5166,7 @@
         <v>34.58831634451302</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>21.84335014545107</v>
+        <v>21.84335020422503</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>1.387556656419027</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.0354636871700866</v>
+        <v>-0.0354636871589564</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>44.39129554813244</v>
+        <v>44.39129573578995</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>18.65092197311215</v>
+        <v>18.65092201139734</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.2464438420817963</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-0.026157243276887</v>
+        <v>-0.026157243221251</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>52.45059471195558</v>
+        <v>52.45059470395751</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>7.012534892348604</v>
+        <v>7.012534931196867</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>1.942153480615019</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.4857290495598072</v>
+        <v>-0.4857290492259927</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>51.57708376091636</v>
+        <v>51.57708315184491</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>4.704783684963662</v>
+        <v>4.704783624617333</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>1.626767920031527</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>0.0026945573673922</v>
+        <v>0.0026945573562677</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>40.78615352195565</v>
+        <v>40.78615390133209</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>10.29199473121068</v>
+        <v>10.29199473202256</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>0.6124963616839333</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>0.0129514751823816</v>
+        <v>0.0129514749598242</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>42.253352349407</v>
+        <v>42.25335317739725</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>14.0030093075931</v>
+        <v>14.00300935627097</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>0.6802068460019411</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.1502917505707335</v>
+        <v>-0.1502917504817166</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>45.36640894271756</v>
+        <v>45.36640895671027</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>15.50505492187771</v>
+        <v>15.50505493219398</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>1.210288978706686</v>
@@ -5520,7 +5520,7 @@
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>289.2171454738008</v>
+        <v>289.2171454738017</v>
       </c>
       <c r="E96" s="2" t="n">
         <v>51.3</v>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>44.89803460419235</v>
+        <v>44.89803461144518</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>10.38640518992784</v>
+        <v>10.38640517914704</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>1.064182859589958</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.1859762703707104</v>
+        <v>0.1859762703484601</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>285.6286989031227</v>
+        <v>285.6286989031228</v>
       </c>
       <c r="E97" s="2" t="n">
         <v>35.25</v>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>42.95399440122907</v>
+        <v>42.95399570442994</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>21.59318462599901</v>
+        <v>21.59318464846947</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>1.183825462344775</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>0.0355931412457075</v>
+        <v>0.0355931411121898</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>41.44635992911208</v>
+        <v>41.4463600159844</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>17.53297212753641</v>
+        <v>17.53297211803904</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.4001806058057411</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.8964715956247549</v>
+        <v>-0.8964715952908993</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>41.30905854479315</v>
+        <v>41.30905866039008</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>36.84329828119234</v>
+        <v>36.8432982995462</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.5356030521272495</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.5176356434261957</v>
+        <v>-0.5176356434484537</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>51.17034121581504</v>
+        <v>51.1703410746649</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>18.94675426563281</v>
+        <v>18.94675435276439</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.5490324118273482</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>0.7958986517877171</v>
+        <v>0.7958986520102493</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>51.88577207117604</v>
+        <v>51.88577207890387</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>8.372005408241936</v>
+        <v>8.372005477334785</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>2.03612805129985</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.2753326640605705</v>
+        <v>-0.275332664116206</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>54.77016665411341</v>
+        <v>54.77016674789161</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>14.42479787258939</v>
+        <v>14.42479787527067</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.3182848225359845</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>0.3530540306306247</v>
+        <v>0.3530540303858229</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5891,7 +5891,7 @@
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>259.273377806105</v>
+        <v>259.2733778061049</v>
       </c>
       <c r="E103" s="2" t="n">
         <v>265</v>
@@ -5905,7 +5905,7 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>41.52148787066806</v>
+        <v>41.52148780532447</v>
       </c>
       <c r="I103" s="2" t="n">
         <v>23.66342085739247</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.2667905237771921</v>
+        <v>-0.2667905235546075</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>38.72294720615293</v>
+        <v>38.72294725942346</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>17.30463057845179</v>
+        <v>17.30463072798693</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>2.590748507323926</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.8472706002441124</v>
+        <v>-0.8472706003553619</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>48.82862204681661</v>
+        <v>48.82862199955958</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>14.16930494877754</v>
+        <v>14.16930491766449</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>1.541350937781964</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.0325565219989162</v>
+        <v>-0.0325565220322996</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>44.54232114396994</v>
+        <v>44.54232162373911</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>22.09569487994574</v>
+        <v>22.09569491402989</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.7393564892775711</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.1265523963576388</v>
+        <v>0.1265523963353877</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6103,7 +6103,7 @@
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>239.4535186733207</v>
+        <v>239.453518673321</v>
       </c>
       <c r="E107" s="2" t="n">
         <v>213.5</v>
@@ -6117,7 +6117,7 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>40.77833486064863</v>
+        <v>40.77833488770919</v>
       </c>
       <c r="I107" s="2" t="n">
         <v>16.28008093910533</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>1.266143435274226</v>
+        <v>1.266143435496769</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6156,7 +6156,7 @@
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>237.4196926294737</v>
+        <v>237.4196926294735</v>
       </c>
       <c r="E108" s="2" t="n">
         <v>62.6</v>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>44.51192901464255</v>
+        <v>44.51192908018325</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>22.3102657160902</v>
+        <v>22.31026571635481</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.6657596540660621</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>0.1063009323047981</v>
+        <v>0.1063009322936709</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>42.02369188243859</v>
+        <v>42.02369193469709</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>31.22547405548758</v>
+        <v>31.22547403096663</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>1.162178652411871</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.0683157384727629</v>
+        <v>-0.0683157384616353</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>44.30469270061081</v>
+        <v>44.30469268736909</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>17.07486363911503</v>
+        <v>17.0748636554645</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>1.054720645528065</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.8857450025403071</v>
+        <v>-0.885745002673846</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>39.85450719741153</v>
+        <v>39.85450718301562</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>18.46706408397181</v>
+        <v>18.46706411518573</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.9725175650890024</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>0.2298632594084009</v>
+        <v>0.2298632593972733</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6368,7 +6368,7 @@
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>219.4083661197825</v>
+        <v>219.4083661197824</v>
       </c>
       <c r="E112" s="2" t="n">
         <v>61.9</v>
@@ -6382,7 +6382,7 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>52.44644401723917</v>
+        <v>52.44644425150198</v>
       </c>
       <c r="I112" s="2" t="n">
         <v>7.997426745756562</v>
@@ -6410,21 +6410,21 @@
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>6560</v>
+        <v>6605</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>欣普羅</t>
+          <t>帝寶</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>217.501900319797</v>
+        <v>218.0190368645028</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>32.8</v>
+        <v>136.5</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,16 +6435,16 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>51.77532948682453</v>
+        <v>47.49986137728362</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>12.24119931831096</v>
+        <v>11.92711674982879</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>1.043739873202432</v>
+        <v>0.3942923313245894</v>
       </c>
       <c r="K113" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L113" s="2" t="n">
         <v>0</v>
@@ -6453,31 +6453,31 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.0173439110471512</v>
+        <v>-0.2222848709266678</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>6515</v>
+        <v>6560</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>穎崴</t>
+          <t>欣普羅</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>216.5743611160392</v>
+        <v>217.5019003197968</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>5615</v>
+        <v>32.8</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,16 +6488,16 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>40.34951319649844</v>
+        <v>51.77532944755421</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>11.93094638888683</v>
+        <v>12.24119936058367</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>1.484203705494706</v>
+        <v>1.043739873202432</v>
       </c>
       <c r="K114" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L114" s="2" t="n">
         <v>0</v>
@@ -6506,31 +6506,31 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-28.79756034549627</v>
+        <v>-0.0173439110471512</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>6720</v>
+        <v>6515</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>久昌</t>
+          <t>穎崴</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>211.3572071733008</v>
+        <v>216.574361116039</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>117</v>
+        <v>5615</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,13 +6541,13 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>45.1906859142774</v>
+        <v>40.34951319551141</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>13.46800521421494</v>
+        <v>11.93094636843228</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>1.981179723012308</v>
+        <v>1.484203705494706</v>
       </c>
       <c r="K115" s="2" t="n">
         <v>1</v>
@@ -6559,31 +6559,31 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.0320069516668106</v>
+        <v>-28.79756034660835</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>6679</v>
+        <v>6720</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>鈺太</t>
+          <t>久昌</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>201.8400682646615</v>
+        <v>211.3572071733015</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>196.5</v>
+        <v>117</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -6594,16 +6594,16 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>41.35313680417778</v>
+        <v>45.19068588516648</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>12.14848856722628</v>
+        <v>13.46800515049276</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>0.8136283136584829</v>
+        <v>1.981179723012308</v>
       </c>
       <c r="K116" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L116" s="2" t="n">
         <v>0</v>
@@ -6612,31 +6612,31 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>0.2229508149708612</v>
+        <v>-0.032006951221732</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>6581</v>
+        <v>6679</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>鋼聯</t>
+          <t>鈺太</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>195.3612913294124</v>
+        <v>201.8400682646615</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>107.5</v>
+        <v>196.5</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -6647,13 +6647,13 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>42.0761403825387</v>
+        <v>41.35313666152096</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>12.88345318986406</v>
+        <v>12.14848856600826</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>0.4998500586134511</v>
+        <v>0.8136283136584829</v>
       </c>
       <c r="K117" s="2" t="n">
         <v>0</v>
@@ -6665,31 +6665,31 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.1692050107087156</v>
+        <v>0.2229508153046757</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>6592</v>
+        <v>6581</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>和潤企業</t>
+          <t>鋼聯</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>185.1829488224045</v>
+        <v>195.3612913294121</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>56.7</v>
+        <v>107.5</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -6700,16 +6700,16 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>35.36866974761246</v>
+        <v>42.07614045875922</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>34.37894275084675</v>
+        <v>12.88345325978941</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>0.552843877341298</v>
+        <v>0.4998500586134511</v>
       </c>
       <c r="K118" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L118" s="2" t="n">
         <v>0</v>
@@ -6718,31 +6718,31 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.1279476707884628</v>
+        <v>-0.1692050109312646</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>6794</v>
+        <v>6592</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>向榮生技-創</t>
+          <t>和潤企業</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>181.3792866838006</v>
+        <v>185.1829488224044</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>71.59999999999999</v>
+        <v>56.7</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -6753,16 +6753,16 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>41.96218918772878</v>
+        <v>35.36866982805408</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>15.11069081978552</v>
+        <v>34.37894269621886</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.8885891172584922</v>
+        <v>0.552843877341298</v>
       </c>
       <c r="K119" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L119" s="2" t="n">
         <v>0</v>
@@ -6771,31 +6771,31 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.262856883699566</v>
+        <v>-0.1279476708107192</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>6680</v>
+        <v>6794</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>鑫創電子</t>
+          <t>向榮生技-創</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>160.0641254566031</v>
+        <v>181.3792866838006</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>0</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -6806,13 +6806,13 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>43.9688102571434</v>
+        <v>41.96218918772878</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>7.202712981477149</v>
+        <v>15.11069082307959</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>0.0146893084628145</v>
+        <v>0.8885891172584922</v>
       </c>
       <c r="K120" s="2" t="n">
         <v>0</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-1.555264194038327</v>
+        <v>-0.2628568837218162</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6834,21 +6834,21 @@
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>6605</v>
+        <v>6680</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>帝寶</t>
+          <t>鑫創電子</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>158.0190368645027</v>
+        <v>160.0641254566031</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>136.5</v>
+        <v>0</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6859,16 +6859,16 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>47.49986135600617</v>
+        <v>43.96881025672404</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>11.92711666588611</v>
+        <v>7.20271293355925</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>0.3942923313245894</v>
+        <v>0.0146893084628145</v>
       </c>
       <c r="K121" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L121" s="2" t="n">
         <v>0</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.2222848702590318</v>
+        <v>-1.555264194216364</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6898,7 +6898,7 @@
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>131.3766682592358</v>
+        <v>131.3766682592343</v>
       </c>
       <c r="E122" s="2" t="n">
         <v>31.6</v>
@@ -6912,10 +6912,10 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>46.98467657335377</v>
+        <v>46.9846764560143</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>12.68355789227464</v>
+        <v>12.68355802767248</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>0.3379481709045224</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.0030590230911952</v>
+        <v>-0.0030590228575272</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6951,7 +6951,7 @@
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>65.97630006752907</v>
+        <v>65.97630006752841</v>
       </c>
       <c r="E123" s="2" t="n">
         <v>73.90000000000001</v>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>42.59115585380086</v>
+        <v>42.591156782979</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>13.88240300096864</v>
+        <v>13.88240286466256</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>0.4372500823207664</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>0.0573295327695932</v>
+        <v>0.0573295319461936</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
scan: seg6 2026-10-10 00:11 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq7_2026-10-08.xlsx
+++ b/output/full_scan/batch_seq7_2026-10-08.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>77.98117717601194</v>
+        <v>77.98117715498653</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>32.15654623362533</v>
+        <v>32.15654622728688</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>4.677801058886754</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>3.628760469858125</v>
+        <v>3.628760469737968</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>74.83919994575774</v>
+        <v>74.83919993124148</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>31.18927914586173</v>
+        <v>31.18927918107638</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>8.986045869853438</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>0.369725636302992</v>
+        <v>0.369725636062645</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>72.28893200630961</v>
+        <v>72.28893207003097</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>34.97202339169168</v>
+        <v>34.97202355779234</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>3.600972489894296</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>2.643565296725784</v>
+        <v>2.643565295524061</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>72.69184569411291</v>
+        <v>72.69184580022306</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>45.21680541636936</v>
+        <v>45.21680547296768</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>1.588509040452033</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>1.844335491300137</v>
+        <v>1.844335489978251</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>61.29899892586664</v>
+        <v>61.29899920851808</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>19.84932217075763</v>
+        <v>19.84932240107641</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>1.958211046203465</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.1140782857706945</v>
+        <v>0.1140782837277387</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>67.31496915714027</v>
+        <v>67.31496915314588</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>43.7761917226742</v>
+        <v>43.77619165520911</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>2.234766192675654</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>1.698063411896504</v>
+        <v>1.698063411956594</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>956.637813742482</v>
+        <v>956.6378137424796</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>61.3</v>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>62.92622639186504</v>
+        <v>62.92622622526066</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>31.60847791229341</v>
+        <v>31.6084781137377</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>5.004460398320227</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.1403973477860597</v>
+        <v>0.1403973485551635</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>78.26489127375122</v>
+        <v>78.26489126864368</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>58.86761669835523</v>
+        <v>58.86761673150925</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>1.407805070964943</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>1.694036728498101</v>
+        <v>1.694036728377926</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>62.05634877219592</v>
+        <v>62.05634861123368</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>23.7213110707453</v>
+        <v>23.72131111274185</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>4.925135988513275</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.0804040784448317</v>
+        <v>0.0804040785650047</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>72.16885568885512</v>
+        <v>72.16885565511703</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>34.46886449653183</v>
+        <v>34.46886448195668</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>0.9899212603935608</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>17.23845899121328</v>
+        <v>17.23845899373678</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>67.04068626206461</v>
+        <v>67.04068615758069</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>49.95145008508936</v>
+        <v>49.95145017250389</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>0.9765676066623864</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>0.1804956500723107</v>
+        <v>0.1804956504688841</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1121,7 +1121,7 @@
         <v/>
       </c>
       <c r="D13" s="2" t="n">
-        <v>839.1880866732723</v>
+        <v>839.1880866732729</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>1130</v>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>60.07551026141745</v>
+        <v>60.0755102604268</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>21.40133734888824</v>
+        <v>21.40133735881879</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>1.558748156782288</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>25.88294477167234</v>
+        <v>25.88294477143205</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>60.98143054996154</v>
+        <v>60.98143053421795</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>34.82024472648525</v>
+        <v>34.82024475200009</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>0.4722500484871325</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>2.933073678262178</v>
+        <v>2.933073678202075</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>59.93141592953386</v>
+        <v>59.93141593314974</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>29.97730848545966</v>
+        <v>29.97730846882907</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>0.4599786403510817</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0.7378369566981888</v>
+        <v>0.7378369567222212</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1280,7 +1280,7 @@
         <v/>
       </c>
       <c r="D16" s="2" t="n">
-        <v>812.0413633490097</v>
+        <v>812.0413633490094</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>57.9</v>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>63.85340557227724</v>
+        <v>63.85340554558281</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>52.76980748079333</v>
+        <v>52.76980746095487</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>0.7579383884849463</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.5398678632856089</v>
+        <v>0.5398678635499934</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>62.45087865496363</v>
+        <v>62.45087863313301</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>37.4251265617586</v>
+        <v>37.42512658273488</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.6671479768843608</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>1.371633378436911</v>
+        <v>1.371633378677252</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>53.74423820228884</v>
+        <v>53.7442383432869</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>16.77141114280965</v>
+        <v>16.77141117427538</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>3.369596032338268</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>1.821047945352711</v>
+        <v>1.821047943790446</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1439,7 +1439,7 @@
         <v/>
       </c>
       <c r="D19" s="2" t="n">
-        <v>784.4836227024335</v>
+        <v>784.4836227024354</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>94.5</v>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>64.71129052355218</v>
+        <v>64.71128992525033</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>21.7000178768023</v>
+        <v>21.7000175128348</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>3.412775877263639</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>0.5595636934888701</v>
+        <v>0.5595636957481189</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>59.92352121230864</v>
+        <v>59.92352121704964</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>28.10003335483679</v>
+        <v>28.10003339919522</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>0.5938275576627133</v>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>58.98838755467104</v>
+        <v>58.9883875571286</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>19.98650739552722</v>
+        <v>19.98650739349332</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>0.9086385847321282</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>0.6291563055438465</v>
+        <v>0.6291563055318437</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
         <v/>
       </c>
       <c r="D22" s="2" t="n">
-        <v>731.9976242804454</v>
+        <v>731.9976242804453</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>34.85</v>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>60.35221769892848</v>
+        <v>60.35221765929589</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>22.91547816282246</v>
+        <v>22.91547829064359</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>0.7168845755629784</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0.054635242231444</v>
+        <v>0.0546352423275858</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>84.81904218199512</v>
+        <v>84.8190424658852</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>39.8756095946842</v>
+        <v>39.87560958061536</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>1.427086274795852</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0.5232259810734681</v>
+        <v>0.5232259807970707</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>57.21265625371881</v>
+        <v>57.21265615739381</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>22.198839170357</v>
+        <v>22.19883938539926</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>1.263692939504653</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.5573243875637813</v>
+        <v>0.557324387780096</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1757,7 +1757,7 @@
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>695.1341194009391</v>
+        <v>695.1341194009392</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>373.5</v>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>57.69248789179114</v>
+        <v>57.6924877023189</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>19.90899441238585</v>
+        <v>19.90899432240124</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0.6487988894853873</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>3.143409793613073</v>
+        <v>3.143409796497235</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>55.89339953111688</v>
+        <v>55.89339954851324</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>45.23997928287091</v>
+        <v>45.23997927707968</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>1.273289781574087</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.3979803101205723</v>
+        <v>0.3979803099523256</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>50.80152832275295</v>
+        <v>50.8015283188108</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>42.73984061532882</v>
+        <v>42.73984061390887</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>2.70371125986594</v>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>62.91383970364562</v>
+        <v>62.91383968825833</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>37.93571629859821</v>
+        <v>37.93571626607466</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>1.81992411117357</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>1.511951910716803</v>
+        <v>1.511951910644687</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>57.31869469677081</v>
+        <v>57.31869469070025</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>51.64979246264099</v>
+        <v>51.64979251085062</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>0.2074449238610302</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>-0.474803591611451</v>
+        <v>-0.4748035917556468</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>63.00320033927046</v>
+        <v>63.00320037766296</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>20.37663348387723</v>
+        <v>20.37663349158889</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>3.292200462809101</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>5.279758642122435</v>
+        <v>5.279758641401363</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>56.78172321453793</v>
+        <v>56.78172318874785</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>24.24039646995633</v>
+        <v>24.2403965333102</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>1.222391606073116</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.0949734366415035</v>
+        <v>0.0949734367136062</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>53.51323021848238</v>
+        <v>53.51323024850377</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>29.13121614428152</v>
+        <v>29.13121622809404</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>1.035954040179551</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-1.002055784524414</v>
+        <v>-1.002055785726133</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2181,7 +2181,7 @@
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>613.3696566014031</v>
+        <v>613.369656601403</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>980</v>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>52.31230419904265</v>
+        <v>52.31230420089682</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>15.24503784538327</v>
+        <v>15.24503797018988</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.9618356769682858</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>2.330839334404953</v>
+        <v>2.330839332842736</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2234,7 +2234,7 @@
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>613.053390065798</v>
+        <v>613.0533900657981</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>481</v>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>55.80179150525545</v>
+        <v>55.8017915471145</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>18.26107891569308</v>
+        <v>18.26107893922937</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0.5812664747528452</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>1.878205608663809</v>
+        <v>1.878205610706723</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>611.5031678694868</v>
+        <v>611.5031678694792</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>25.1</v>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>52.93022559344925</v>
+        <v>52.93022491056268</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>25.70036353326663</v>
+        <v>25.70036388702493</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.6387597636512786</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.1453812940973958</v>
+        <v>0.1453812948424661</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2340,7 +2340,7 @@
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>601.7307962642836</v>
+        <v>601.7307962642838</v>
       </c>
       <c r="E36" s="2" t="n">
         <v>96.09999999999999</v>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>50.31989693771708</v>
+        <v>50.31989685855665</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>31.21094350049081</v>
+        <v>31.21094351302317</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.4090974794755025</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-0.923050468100402</v>
+        <v>-0.923050468004269</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2393,7 +2393,7 @@
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>598.4885307453978</v>
+        <v>598.4885307453977</v>
       </c>
       <c r="E37" s="2" t="n">
         <v>3320</v>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>54.38830474779282</v>
+        <v>54.38830472360577</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>20.54630192904309</v>
+        <v>20.54630194476558</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>1.474164731532992</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>-38.65873843399758</v>
+        <v>-38.65873842318159</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>55.74044001556322</v>
+        <v>55.74043950816912</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>22.01416930767322</v>
+        <v>22.01416938173734</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.2994834962647691</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>0.8141755920302727</v>
+        <v>0.8141755920062386</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>70.10524096242435</v>
+        <v>70.10524142195835</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>39.87952354928882</v>
+        <v>39.87952376751926</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.2721303613979708</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>0.0660485988888147</v>
+        <v>0.0660485987085541</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>54.44282154055057</v>
+        <v>54.44282145542765</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>35.68922857887784</v>
+        <v>35.68922856407466</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>1.034954254007886</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>-17.77727502969026</v>
+        <v>-17.77727501767289</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>66.94144622262783</v>
+        <v>66.94144620095125</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>33.976293537517</v>
+        <v>33.97629347171573</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.9702302192733628</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0.70574479069169</v>
+        <v>0.7057447902350447</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>49.69337066999818</v>
+        <v>49.69337063633709</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>23.60458249324902</v>
+        <v>23.60458245708457</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.4012323580511459</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-5.509054300153176</v>
+        <v>-5.509054298590931</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2728,7 +2728,7 @@
         <v>54.23871078293885</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>34.7761110393562</v>
+        <v>34.77611107259797</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.4059126960222002</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>0.4189830296948678</v>
+        <v>0.4189830284931304</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2764,7 +2764,7 @@
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>546.2834860411032</v>
+        <v>546.2834860411219</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>32.05</v>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>60.39992765887241</v>
+        <v>60.3999276403206</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>20.71831704960949</v>
+        <v>20.71831706782324</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.76842308365379</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.1499796471914191</v>
+        <v>0.1499796472515077</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2817,7 +2817,7 @@
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>543.3948795508323</v>
+        <v>543.3948795508326</v>
       </c>
       <c r="E45" s="2" t="n">
         <v>51.3</v>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>53.33818508233588</v>
+        <v>53.33818513681837</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>21.3153523464286</v>
+        <v>21.31535251348915</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.5655523515812341</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-0.1159263832261293</v>
+        <v>-0.1159263834664711</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>52.02230678844378</v>
+        <v>52.02230678730019</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>11.1130816851763</v>
+        <v>11.11308169083232</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>2.418127818287665</v>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>51.56681841409393</v>
+        <v>51.56681843603696</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>17.15662840939718</v>
+        <v>17.15662839386752</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>2.372104056297936</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.0356306631393133</v>
+        <v>0.0356306630311585</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>50.90533411562049</v>
+        <v>50.90533408349435</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>11.92475909126024</v>
+        <v>11.9247592338984</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>2.690725197121355</v>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>31.69496352542404</v>
+        <v>31.69494290248666</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>32.59382456590205</v>
+        <v>32.59382456590206</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>2.013053626871306</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.4112815436474344</v>
+        <v>0.4112814278470682</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>51.97356043739259</v>
+        <v>51.97356044405408</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>25.3857206679741</v>
+        <v>25.38572067524273</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.3049131851882646</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>0.0996167198419399</v>
+        <v>0.0996167196256285</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3135,7 +3135,7 @@
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>525.0919410113352</v>
+        <v>525.0919410113355</v>
       </c>
       <c r="E51" s="2" t="n">
         <v>42.7</v>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>59.58064851185962</v>
+        <v>59.58064843441741</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>19.58274036768908</v>
+        <v>19.58274037491755</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>1.384728293230064</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-0.0258894578383286</v>
+        <v>-0.0258894577421916</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>48.30777085804998</v>
+        <v>48.30777088014377</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>20.42390699357122</v>
+        <v>20.42390698028316</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.3048159697488382</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-0.9461648875038152</v>
+        <v>-0.9461648875398608</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>44.60397899676303</v>
+        <v>44.6039790008111</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>20.06361044251097</v>
+        <v>20.06361050667923</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>1.657099006575845</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-0.0183815861758046</v>
+        <v>-0.0183815862719491</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3294,7 +3294,7 @@
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>516.541191612517</v>
+        <v>516.5411916125165</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>34</v>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>52.12373603468044</v>
+        <v>52.12373603325366</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>12.51999809700345</v>
+        <v>12.51999813933193</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>4.697438928066099</v>
@@ -3347,7 +3347,7 @@
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>499.8940287804564</v>
+        <v>499.894028780456</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>31.8</v>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>55.58318128188915</v>
+        <v>55.58318121784156</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>13.61404865239989</v>
+        <v>13.61404862953015</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>2.522669972002799</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.0809028410406602</v>
+        <v>0.080902841088727</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>52.08940430090089</v>
+        <v>52.08940429753648</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>8.136581882106729</v>
+        <v>8.136581857372251</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.6762794966548318</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.1599916666871392</v>
+        <v>0.1599916666991551</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3453,7 +3453,7 @@
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>497.7344371837373</v>
+        <v>497.7344371837374</v>
       </c>
       <c r="E57" s="2" t="n">
         <v>308.5</v>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>39.43794979259269</v>
+        <v>39.43795003768385</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>20.72798244324854</v>
+        <v>20.72798228439279</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>1.787865829468616</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.3012250305823132</v>
+        <v>0.301225030462148</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>51.50018067503167</v>
+        <v>51.50018057147671</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>14.47981322996224</v>
+        <v>14.47981321877516</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>1.258746950402002</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.4586355738945528</v>
+        <v>0.458635573942625</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>56.76519303941593</v>
+        <v>56.76519300448015</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>35.59071161988214</v>
+        <v>35.5907116993121</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>0.3036177039866246</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.5808116651343025</v>
+        <v>-0.5808116654948292</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3612,7 +3612,7 @@
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>450.3698303674955</v>
+        <v>450.3698303674956</v>
       </c>
       <c r="E60" s="2" t="n">
         <v>210</v>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>46.44390463852518</v>
+        <v>46.44390459580998</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>10.22681481625967</v>
+        <v>10.22681483438185</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.4974877860698913</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.4033154453440959</v>
+        <v>-0.4033154451037424</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3665,7 +3665,7 @@
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>445.2297543505237</v>
+        <v>445.2297543505236</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>53</v>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>54.94998433308984</v>
+        <v>54.94998437920296</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>12.37374604800107</v>
+        <v>12.37374595570635</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.7058512164653069</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.1118318260248105</v>
+        <v>0.1118318259286699</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>42.65358391383797</v>
+        <v>42.65358369998252</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>16.43027833260744</v>
+        <v>16.43027842888686</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.4514499282606705</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.017619246838868</v>
+        <v>0.0176192469590404</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3771,7 +3771,7 @@
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>444.0379372480064</v>
+        <v>444.0379372480061</v>
       </c>
       <c r="E63" s="2" t="n">
         <v>138</v>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>52.46872791315004</v>
+        <v>52.46872787849292</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>14.33720508707962</v>
+        <v>14.3372050716058</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.9173885250808316</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>1.306738551711339</v>
+        <v>1.306738551807484</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>71.4529838752851</v>
+        <v>71.4529842502874</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>33.66978099130186</v>
+        <v>33.66978099104023</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.6454769209701262</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.4994493591701809</v>
+        <v>0.4994493590748321</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>49.87765930767628</v>
+        <v>49.87765929616457</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>13.34529036475397</v>
+        <v>13.34529037385137</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.9913914097643453</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-0.1256714282195001</v>
+        <v>-0.1256714281473931</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>48.63256502103121</v>
+        <v>48.6325650822402</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>16.96765016338534</v>
+        <v>16.9676502444618</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.4202645054255581</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-1.896940139632627</v>
+        <v>-1.896940140714209</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3983,7 +3983,7 @@
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>427.7459199084135</v>
+        <v>427.7459199084136</v>
       </c>
       <c r="E67" s="2" t="n">
         <v>1050</v>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>45.53960811224642</v>
+        <v>45.53960814654408</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>19.3493563504213</v>
+        <v>19.34935634510578</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.4803562824736629</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-5.711683043636535</v>
+        <v>-5.711683044838197</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>32.04679708368592</v>
+        <v>32.04679699751671</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>44.11891517530357</v>
+        <v>44.11891513366643</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.6863659101217567</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>148.6955938158051</v>
+        <v>148.6955938350329</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4089,7 +4089,7 @@
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>422.9168282810193</v>
+        <v>422.9168282810194</v>
       </c>
       <c r="E69" s="2" t="n">
         <v>99.2</v>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>32.77380206114455</v>
+        <v>32.77380202659248</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>32.08668489455518</v>
+        <v>32.08668496286717</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>4.026592479560937</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.1379847763039099</v>
+        <v>0.1379847763519932</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4142,7 +4142,7 @@
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>402.6555650695767</v>
+        <v>402.6555650695765</v>
       </c>
       <c r="E70" s="2" t="n">
         <v>54.2</v>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>31.7977173726148</v>
+        <v>31.79771740420482</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>29.14830981818112</v>
+        <v>29.14830992332267</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>1.73602479466562</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.3452199761043486</v>
+        <v>-0.345219976344699</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4195,7 +4195,7 @@
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>399.6809458718973</v>
+        <v>399.6809458718941</v>
       </c>
       <c r="E71" s="2" t="n">
         <v>44.9</v>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>59.3099726755714</v>
+        <v>59.30997279744708</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>27.58468502559269</v>
+        <v>27.58468515211698</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.4062291653049218</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.5978495108324979</v>
+        <v>0.5978495104719814</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4248,7 +4248,7 @@
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>398.8761491707783</v>
+        <v>398.8761491707781</v>
       </c>
       <c r="E72" s="2" t="n">
         <v>48.05</v>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>48.7185649513577</v>
+        <v>48.71856493334558</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>26.72206878919548</v>
+        <v>26.72206882145424</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.321676861844581</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.0276593456994057</v>
+        <v>-0.0276593460118566</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4301,7 +4301,7 @@
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>379.610644196564</v>
+        <v>379.6106441965641</v>
       </c>
       <c r="E73" s="2" t="n">
         <v>73.5</v>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>56.7869892741137</v>
+        <v>56.78698922895951</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>18.62629727608011</v>
+        <v>18.62629730293778</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.9010651670525968</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>1.208408950024259</v>
+        <v>1.208408949543576</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>372.3149657976858</v>
+        <v>372.3149657976857</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>63.8</v>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>50.2399688689736</v>
+        <v>50.23996902826247</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>21.76144599795549</v>
+        <v>21.76144583795996</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.6924347398800291</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.3768378602593487</v>
+        <v>0.3768378592979646</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>46.43350865589453</v>
+        <v>46.43350816383153</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>9.95346746950699</v>
+        <v>9.953467559790914</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>1.114669928673481</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>3.399155882860882</v>
+        <v>3.399155900886869</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>43.93109224022478</v>
+        <v>43.93109226472005</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>17.17684093117329</v>
+        <v>17.1768407704374</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.5066068051551553</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>0.0347559546232736</v>
+        <v>0.0347559548371809</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4513,7 +4513,7 @@
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>370.2800374495285</v>
+        <v>370.2800374495284</v>
       </c>
       <c r="E77" s="2" t="n">
         <v>97.59999999999999</v>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>49.146285629745</v>
+        <v>49.14628545766488</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>14.23185934882007</v>
+        <v>14.23185934100966</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>1.082389298403912</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.0431989906704554</v>
+        <v>0.0431989909108007</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4566,7 +4566,7 @@
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>369.4835233867393</v>
+        <v>369.4835233867375</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>476</v>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>35.74053652099506</v>
+        <v>35.74053650242223</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>24.98249145296979</v>
+        <v>24.9824914482443</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>2.2835170369843</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.943139429560386</v>
+        <v>0.9431394298007733</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4619,7 +4619,7 @@
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>366.328621165777</v>
+        <v>366.3286211657771</v>
       </c>
       <c r="E79" s="2" t="n">
         <v>62.6</v>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>45.72344533501381</v>
+        <v>45.723445287972</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>22.91381087841981</v>
+        <v>22.91381084756886</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.112792326522207</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.3960621071361779</v>
+        <v>-0.3960621073284511</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4672,7 +4672,7 @@
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>356.1528024815327</v>
+        <v>356.1528024815353</v>
       </c>
       <c r="E80" s="2" t="n">
         <v>41.8</v>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>40.42784782528297</v>
+        <v>40.42784808319156</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>28.2648153374927</v>
+        <v>28.26481534088063</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.4459724409744567</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-0.1123719555735493</v>
+        <v>-0.1123719555014485</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4725,7 +4725,7 @@
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>354.4122186118169</v>
+        <v>354.412218611815</v>
       </c>
       <c r="E81" s="2" t="n">
         <v>1080</v>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>47.17907481520366</v>
+        <v>47.1790748177068</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>10.4450300044397</v>
+        <v>10.44503005117853</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.4386535314835921</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-5.777790601948931</v>
+        <v>-5.777790598223502</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>49.97945205825455</v>
+        <v>49.97945217551752</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>11.84312293151415</v>
+        <v>11.84312309342045</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>0.4282696609609741</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.1079734457719877</v>
+        <v>0.1079734456518139</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4831,7 +4831,7 @@
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>349.9893876942696</v>
+        <v>349.9893876942695</v>
       </c>
       <c r="E83" s="2" t="n">
         <v>24.5</v>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>48.93378349139741</v>
+        <v>48.93378389682966</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>17.03167715970389</v>
+        <v>17.0316772114118</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.5063964740271319</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.0718074553792336</v>
+        <v>0.0718074556436147</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>50.36687054060497</v>
+        <v>50.36687059641377</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>6.867971449404723</v>
+        <v>6.867971476444219</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>1.23093580121998</v>
@@ -4937,7 +4937,7 @@
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>337.5790327226318</v>
+        <v>337.5790327226375</v>
       </c>
       <c r="E85" s="2" t="n">
         <v>41.55</v>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>52.02671497220875</v>
+        <v>52.02671479235777</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>17.52343362253448</v>
+        <v>17.52343361634577</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>0.7005465057417336</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>0.0694930730474904</v>
+        <v>0.0694930730955539</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -4990,7 +4990,7 @@
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>336.2429150946988</v>
+        <v>336.2429150946991</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>1415</v>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>47.65097970079854</v>
+        <v>47.65097968357654</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>16.8332625949138</v>
+        <v>16.83326248028898</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.4293236982277061</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-22.49594668619365</v>
+        <v>-22.49594668054547</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>46.65280283291249</v>
+        <v>46.65280250658098</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>13.43740418864064</v>
+        <v>13.4374042083838</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.6148936400018552</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.5909126842931918</v>
+        <v>0.5909126870571484</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>50.18046394032337</v>
+        <v>50.18046391218545</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>23.36733376986713</v>
+        <v>23.36733377628344</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>1.057565219358469</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.06978578344767331</v>
+        <v>0.0697857833755702</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5149,7 +5149,7 @@
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>305.2659183361569</v>
+        <v>305.2659183361568</v>
       </c>
       <c r="E89" s="2" t="n">
         <v>37.25</v>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>34.58831634451302</v>
+        <v>34.58831627725891</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>21.84335020422503</v>
+        <v>21.84335021711794</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>1.387556656419027</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.0354636871589564</v>
+        <v>-0.0354636871469424</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>44.39129573578995</v>
+        <v>44.39129541970608</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>18.65092201139734</v>
+        <v>18.65092190981676</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.2464438420817963</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-0.026157243221251</v>
+        <v>-0.0261572426804739</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5272,7 +5272,7 @@
         <v>52.45059470395751</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>7.012534931196867</v>
+        <v>7.012534863436247</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>1.942153480615019</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.4857290492259927</v>
+        <v>-0.4857290495865198</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>51.57708315184491</v>
+        <v>51.57708443156477</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>4.704783624617333</v>
+        <v>4.704784389770527</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>1.626767920031527</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>0.0026945573562677</v>
+        <v>0.0026945489441563</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>40.78615390133209</v>
+        <v>40.78615349277285</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>10.29199473202256</v>
+        <v>10.2919947457128</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>0.6124963616839333</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>0.0129514749598242</v>
+        <v>0.0129514765220672</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>42.25335317739725</v>
+        <v>42.25335220276828</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>14.00300935627097</v>
+        <v>14.00300973159179</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>0.6802068460019411</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.1502917504817166</v>
+        <v>-0.1502917493520929</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>45.36640895671027</v>
+        <v>45.3664089416412</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>15.50505493219398</v>
+        <v>15.5050549167498</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>1.210288978706686</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>0.09123580417530031</v>
+        <v>0.0912358042954737</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5520,7 +5520,7 @@
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>289.2171454738017</v>
+        <v>289.2171454738008</v>
       </c>
       <c r="E96" s="2" t="n">
         <v>51.3</v>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>44.89803461144518</v>
+        <v>44.89803462582395</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>10.38640517914704</v>
+        <v>10.3864053128012</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>1.064182859589958</v>
@@ -5573,7 +5573,7 @@
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>285.6286989031228</v>
+        <v>285.6286989031224</v>
       </c>
       <c r="E97" s="2" t="n">
         <v>35.25</v>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>42.95399570442994</v>
+        <v>42.95399636646559</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>21.59318464846947</v>
+        <v>21.59318478163772</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>1.183825462344775</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>0.0355931411121898</v>
+        <v>0.0355931420735725</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>41.4463600159844</v>
+        <v>41.44635988054813</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>17.53297211803904</v>
+        <v>17.53297212768585</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.4001806058057411</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.8964715952908993</v>
+        <v>-0.896471591084838</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>41.30905866039008</v>
+        <v>41.30905869229986</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>36.8432982995462</v>
+        <v>36.84329817956474</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.5356030521272495</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.5176356434484537</v>
+        <v>-0.5176356431840607</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>51.1703410746649</v>
+        <v>51.17034114067382</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>18.94675435276439</v>
+        <v>18.9467544273012</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.5490324118273482</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>0.7958986520102493</v>
+        <v>0.7958986514094157</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>51.88577207890387</v>
+        <v>51.88577207307595</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>8.372005477334785</v>
+        <v>8.372005493935355</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>2.03612805129985</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.275332664116206</v>
+        <v>-0.2753326640080536</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5838,7 +5838,7 @@
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>263.7078329186533</v>
+        <v>263.7078329186534</v>
       </c>
       <c r="E102" s="2" t="n">
         <v>61.5</v>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>54.77016674789161</v>
+        <v>54.77016660650295</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>14.42479787527067</v>
+        <v>14.4247979138631</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.3182848225359845</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>0.3530540303858229</v>
+        <v>0.3530540303617901</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>41.52148780532447</v>
+        <v>41.52148775535967</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>23.66342085739247</v>
+        <v>23.66342086629992</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.9871368359664936</v>
@@ -5944,7 +5944,7 @@
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>253.1065141044332</v>
+        <v>253.106514104438</v>
       </c>
       <c r="E104" s="2" t="n">
         <v>129</v>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>38.72294725942346</v>
+        <v>38.72294717857503</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>17.30463072798693</v>
+        <v>17.30463072792977</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>2.590748507323926</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.8472706003553619</v>
+        <v>-0.8472705998746699</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -5997,7 +5997,7 @@
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>240.5529900093201</v>
+        <v>240.5529900093202</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>41.5</v>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>48.82862199955958</v>
+        <v>48.82862192322128</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>14.16930491766449</v>
+        <v>14.16930490314349</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>1.541350937781964</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.0325565220322996</v>
+        <v>-0.0325565221644937</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>44.54232162373911</v>
+        <v>44.54232093063666</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>22.09569491402989</v>
+        <v>22.09569499154428</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.7393564892775711</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.1265523963353877</v>
+        <v>0.1265523977293948</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6103,7 +6103,7 @@
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>239.453518673321</v>
+        <v>239.4535186733208</v>
       </c>
       <c r="E107" s="2" t="n">
         <v>213.5</v>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>40.77833488770919</v>
+        <v>40.77833505284802</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>16.28008093910533</v>
+        <v>16.28008099183922</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>1.664168467255676</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>1.266143435496769</v>
+        <v>1.266143436097624</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>44.51192908018325</v>
+        <v>44.51192900960096</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>22.31026571635481</v>
+        <v>22.3102657251978</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.6657596540660621</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>0.1063009322936709</v>
+        <v>0.106300932570056</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>42.02369193469709</v>
+        <v>42.02369181005289</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>31.22547403096663</v>
+        <v>31.2254739485601</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>1.162178652411871</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.0683157384616353</v>
+        <v>-0.0683157383895318</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6262,7 +6262,7 @@
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>229.8581927843686</v>
+        <v>229.8581927843685</v>
       </c>
       <c r="E110" s="2" t="n">
         <v>141.5</v>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>44.30469268736909</v>
+        <v>44.30469270004493</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>17.0748636554645</v>
+        <v>17.07486381338252</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>1.054720645528065</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.885745002673846</v>
+        <v>-0.8857450030343355</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>39.85450718301562</v>
+        <v>39.85450717784787</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>18.46706411518573</v>
+        <v>18.46706411807941</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.9725175650890024</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>0.2298632593972733</v>
+        <v>0.2298632593492047</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>52.44644425150198</v>
+        <v>52.44644374880208</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>7.997426745756562</v>
+        <v>7.997426784707299</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.4710328832803629</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.1343614052586068</v>
+        <v>0.1343614057392905</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>47.49986137728362</v>
+        <v>47.49986135436945</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>11.92711674982879</v>
+        <v>11.92711676405301</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.3942923313245894</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.2222848709266678</v>
+        <v>-0.2222848715275329</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>51.77532944755421</v>
+        <v>51.77532947134296</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>12.24119936058367</v>
+        <v>12.24119960655522</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>1.043739873202432</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.0173439110471512</v>
+        <v>-0.0173439112394323</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6527,7 +6527,7 @@
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>216.574361116039</v>
+        <v>216.5743611160387</v>
       </c>
       <c r="E115" s="2" t="n">
         <v>5615</v>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>40.34951319551141</v>
+        <v>40.34951319232254</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>11.93094636843228</v>
+        <v>11.93094642242114</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>1.484203705494706</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-28.79756034660835</v>
+        <v>-28.79756034901214</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6580,7 +6580,7 @@
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>211.3572071733015</v>
+        <v>211.3572071733013</v>
       </c>
       <c r="E116" s="2" t="n">
         <v>117</v>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>45.19068588516648</v>
+        <v>45.19068589714535</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>13.46800515049276</v>
+        <v>13.46800504560437</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>1.981179723012308</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.032006951221732</v>
+        <v>-0.0320069515822525</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6633,7 +6633,7 @@
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>201.8400682646615</v>
+        <v>201.8400682646614</v>
       </c>
       <c r="E117" s="2" t="n">
         <v>196.5</v>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>41.35313666152096</v>
+        <v>41.35313674165464</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>12.14848856600826</v>
+        <v>12.14848859705719</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>0.8136283136584829</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>0.2229508153046757</v>
+        <v>0.2229508137424194</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>42.07614045875922</v>
+        <v>42.07614057175916</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>12.88345325978941</v>
+        <v>12.88345337740648</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>0.4998500586134511</v>
@@ -6739,7 +6739,7 @@
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>185.1829488224044</v>
+        <v>185.1829488224045</v>
       </c>
       <c r="E119" s="2" t="n">
         <v>56.7</v>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>35.36866982805408</v>
+        <v>35.3686697101484</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>34.37894269621886</v>
+        <v>34.37894255931971</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>0.552843877341298</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.1279476708107192</v>
+        <v>-0.1279476707145832</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>41.96218918772878</v>
+        <v>41.96218916585919</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>15.11069082307959</v>
+        <v>15.1106908248091</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>0.8885891172584922</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.2628568837218162</v>
+        <v>-0.2628568837458487</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>43.96881025672404</v>
+        <v>43.96881025898214</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>7.20271293355925</v>
+        <v>7.202712943215906</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>0.0146893084628145</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-1.555264194216364</v>
+        <v>-1.55526419445671</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6898,7 +6898,7 @@
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>131.3766682592343</v>
+        <v>131.376668259235</v>
       </c>
       <c r="E122" s="2" t="n">
         <v>31.6</v>
@@ -6912,10 +6912,10 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>46.9846764560143</v>
+        <v>46.98467637414289</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>12.68355802767248</v>
+        <v>12.68355806128125</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>0.3379481709045224</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.0030590228575272</v>
+        <v>-0.0030590228695506</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6951,7 +6951,7 @@
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>65.97630006752841</v>
+        <v>65.97630006752864</v>
       </c>
       <c r="E123" s="2" t="n">
         <v>73.90000000000001</v>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>42.591156782979</v>
+        <v>42.59115663840577</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>13.88240286466256</v>
+        <v>13.88240279738144</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>0.4372500823207664</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>0.0573295319461936</v>
+        <v>0.0573295324509057</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>

</xml_diff>